<commit_message>
Implement Project Insights page, Matrix Comparison table, and UI refinements
</commit_message>
<xml_diff>
--- a/backend/rankings.xlsx
+++ b/backend/rankings.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4538" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4628" uniqueCount="372">
   <si>
     <t>Keyword / Date</t>
   </si>
@@ -1121,6 +1121,21 @@
   </si>
   <si>
     <t>1//6 LL 4</t>
+  </si>
+  <si>
+    <t>1//7 LL 1</t>
+  </si>
+  <si>
+    <t>1//1 LL 7</t>
+  </si>
+  <si>
+    <t>1//1 LL 2</t>
+  </si>
+  <si>
+    <t>2026-04-30</t>
+  </si>
+  <si>
+    <t>1//8 LL 8</t>
   </si>
 </sst>
 </file>
@@ -1588,7 +1603,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -1742,9 +1757,339 @@
         <v>363</v>
       </c>
     </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>106</v>
+      </c>
+      <c r="C14" t="s">
+        <v>367</v>
+      </c>
+      <c r="D14" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>110</v>
+      </c>
+      <c r="C15" t="s">
+        <v>95</v>
+      </c>
+      <c r="D15" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>110</v>
+      </c>
+      <c r="C16" t="s">
+        <v>95</v>
+      </c>
+      <c r="D16" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>112</v>
+      </c>
+      <c r="C17" t="s">
+        <v>64</v>
+      </c>
+      <c r="D17" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>110</v>
+      </c>
+      <c r="C18" t="s">
+        <v>95</v>
+      </c>
+      <c r="D18" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>112</v>
+      </c>
+      <c r="C19" t="s">
+        <v>368</v>
+      </c>
+      <c r="D19" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>114</v>
+      </c>
+      <c r="C20" t="s">
+        <v>75</v>
+      </c>
+      <c r="D20" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>108</v>
+      </c>
+      <c r="C21" t="s">
+        <v>75</v>
+      </c>
+      <c r="D21" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>110</v>
+      </c>
+      <c r="C22" t="s">
+        <v>19</v>
+      </c>
+      <c r="D22" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>116</v>
+      </c>
+      <c r="C23" t="s">
+        <v>30</v>
+      </c>
+      <c r="D23" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>104</v>
+      </c>
+      <c r="C24" t="s">
+        <v>64</v>
+      </c>
+      <c r="D24" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>104</v>
+      </c>
+      <c r="C25" t="s">
+        <v>64</v>
+      </c>
+      <c r="D25" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>104</v>
+      </c>
+      <c r="C26" t="s">
+        <v>64</v>
+      </c>
+      <c r="D26" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>104</v>
+      </c>
+      <c r="C27" t="s">
+        <v>369</v>
+      </c>
+      <c r="D27" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>104</v>
+      </c>
+      <c r="C28" t="s">
+        <v>64</v>
+      </c>
+      <c r="D28" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>106</v>
+      </c>
+      <c r="C29" t="s">
+        <v>64</v>
+      </c>
+      <c r="D29" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>108</v>
+      </c>
+      <c r="C30" t="s">
+        <v>75</v>
+      </c>
+      <c r="D30" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>110</v>
+      </c>
+      <c r="C31" t="s">
+        <v>37</v>
+      </c>
+      <c r="D31" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>112</v>
+      </c>
+      <c r="C32" t="s">
+        <v>97</v>
+      </c>
+      <c r="D32" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>114</v>
+      </c>
+      <c r="C33" t="s">
+        <v>97</v>
+      </c>
+      <c r="D33" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>116</v>
+      </c>
+      <c r="C34" t="s">
+        <v>75</v>
+      </c>
+      <c r="D34" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>118</v>
+      </c>
+      <c r="C35" t="s">
+        <v>64</v>
+      </c>
+      <c r="D35" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>120</v>
+      </c>
+      <c r="C36" t="s">
+        <v>19</v>
+      </c>
+      <c r="D36" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>122</v>
+      </c>
+      <c r="C37" t="s">
+        <v>364</v>
+      </c>
+      <c r="D37" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>124</v>
+      </c>
+      <c r="C38" t="s">
+        <v>19</v>
+      </c>
+      <c r="D38" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>126</v>
+      </c>
+      <c r="C39" t="s">
+        <v>15</v>
+      </c>
+      <c r="D39" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>126</v>
+      </c>
+      <c r="C40" t="s">
+        <v>371</v>
+      </c>
+      <c r="D40" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>112</v>
+      </c>
+      <c r="C41" t="s">
+        <v>368</v>
+      </c>
+      <c r="D41" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>122</v>
+      </c>
+      <c r="C42" t="s">
+        <v>75</v>
+      </c>
+      <c r="D42" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>122</v>
+      </c>
+      <c r="C43" t="s">
+        <v>364</v>
+      </c>
+      <c r="D43" t="s">
+        <v>370</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
🚀 LIVE DEPLOYMENT: Rebranded to Ranking Anywhere and configured production URLs
</commit_message>
<xml_diff>
--- a/backend/rankings.xlsx
+++ b/backend/rankings.xlsx
@@ -14,13 +14,14 @@
     <sheet sheetId="8" name="are-corp.com" state="visible" r:id="rId11"/>
     <sheet sheetId="9" name="abc.con" state="visible" r:id="rId12"/>
     <sheet sheetId="10" name="adamdental.com.au" state="visible" r:id="rId13"/>
+    <sheet sheetId="11" name="challengebricksandroofing.com.a" state="visible" r:id="rId14"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4628" uniqueCount="372">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4917" uniqueCount="389">
   <si>
     <t>Keyword / Date</t>
   </si>
@@ -1136,6 +1137,57 @@
   </si>
   <si>
     <t>1//8 LL 8</t>
+  </si>
+  <si>
+    <t>2026-05-01</t>
+  </si>
+  <si>
+    <t>1//2 LL 7</t>
+  </si>
+  <si>
+    <t>1//3 LL 4</t>
+  </si>
+  <si>
+    <t>2026-05-03</t>
+  </si>
+  <si>
+    <t>1//2 LL 10</t>
+  </si>
+  <si>
+    <t>velux skylight installation near me</t>
+  </si>
+  <si>
+    <t>velux skylights melbourne</t>
+  </si>
+  <si>
+    <t>velux skylight installation melbourne</t>
+  </si>
+  <si>
+    <t>austral bricks melbourne</t>
+  </si>
+  <si>
+    <t>pgh bricks melbourne</t>
+  </si>
+  <si>
+    <t>monier roof tiles melbourne</t>
+  </si>
+  <si>
+    <t>re roofing melbourne</t>
+  </si>
+  <si>
+    <t>roof replacements melbourne</t>
+  </si>
+  <si>
+    <t>roof replacements near me</t>
+  </si>
+  <si>
+    <t>roof restoration dandenong</t>
+  </si>
+  <si>
+    <t xml:space="preserve">roof restoration berwick </t>
+  </si>
+  <si>
+    <t>roof restoration cranbourne</t>
   </si>
 </sst>
 </file>
@@ -1603,7 +1655,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D79"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -2085,6 +2137,1081 @@
       </c>
       <c r="D43" t="s">
         <v>370</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>104</v>
+      </c>
+      <c r="C44" t="s">
+        <v>369</v>
+      </c>
+      <c r="D44" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>106</v>
+      </c>
+      <c r="C45" t="s">
+        <v>67</v>
+      </c>
+      <c r="D45" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>108</v>
+      </c>
+      <c r="C46" t="s">
+        <v>97</v>
+      </c>
+      <c r="D46" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>110</v>
+      </c>
+      <c r="C47" t="s">
+        <v>19</v>
+      </c>
+      <c r="D47" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>112</v>
+      </c>
+      <c r="C48" t="s">
+        <v>373</v>
+      </c>
+      <c r="D48" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>114</v>
+      </c>
+      <c r="C49" t="s">
+        <v>37</v>
+      </c>
+      <c r="D49" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>116</v>
+      </c>
+      <c r="C50" t="s">
+        <v>75</v>
+      </c>
+      <c r="D50" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>118</v>
+      </c>
+      <c r="C51" t="s">
+        <v>64</v>
+      </c>
+      <c r="D51" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>120</v>
+      </c>
+      <c r="C52" t="s">
+        <v>16</v>
+      </c>
+      <c r="D52" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>122</v>
+      </c>
+      <c r="C53" t="s">
+        <v>364</v>
+      </c>
+      <c r="D53" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>124</v>
+      </c>
+      <c r="C54" t="s">
+        <v>19</v>
+      </c>
+      <c r="D54" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>126</v>
+      </c>
+      <c r="C55" t="s">
+        <v>374</v>
+      </c>
+      <c r="D55" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>104</v>
+      </c>
+      <c r="C56" t="s">
+        <v>3</v>
+      </c>
+      <c r="D56" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>106</v>
+      </c>
+      <c r="C57" t="s">
+        <v>3</v>
+      </c>
+      <c r="D57" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>108</v>
+      </c>
+      <c r="C58" t="s">
+        <v>3</v>
+      </c>
+      <c r="D58" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>110</v>
+      </c>
+      <c r="C59" t="s">
+        <v>3</v>
+      </c>
+      <c r="D59" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>112</v>
+      </c>
+      <c r="C60" t="s">
+        <v>3</v>
+      </c>
+      <c r="D60" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>114</v>
+      </c>
+      <c r="C61" t="s">
+        <v>3</v>
+      </c>
+      <c r="D61" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>116</v>
+      </c>
+      <c r="C62" t="s">
+        <v>3</v>
+      </c>
+      <c r="D62" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>118</v>
+      </c>
+      <c r="C63" t="s">
+        <v>3</v>
+      </c>
+      <c r="D63" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>120</v>
+      </c>
+      <c r="C64" t="s">
+        <v>3</v>
+      </c>
+      <c r="D64" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>122</v>
+      </c>
+      <c r="C65" t="s">
+        <v>3</v>
+      </c>
+      <c r="D65" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>124</v>
+      </c>
+      <c r="C66" t="s">
+        <v>3</v>
+      </c>
+      <c r="D66" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>126</v>
+      </c>
+      <c r="C67" t="s">
+        <v>3</v>
+      </c>
+      <c r="D67" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>104</v>
+      </c>
+      <c r="C68" t="s">
+        <v>369</v>
+      </c>
+      <c r="D68" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>106</v>
+      </c>
+      <c r="C69" t="s">
+        <v>67</v>
+      </c>
+      <c r="D69" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>108</v>
+      </c>
+      <c r="C70" t="s">
+        <v>97</v>
+      </c>
+      <c r="D70" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>108</v>
+      </c>
+      <c r="C71" t="s">
+        <v>97</v>
+      </c>
+      <c r="D71" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>110</v>
+      </c>
+      <c r="C72" t="s">
+        <v>19</v>
+      </c>
+      <c r="D72" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>112</v>
+      </c>
+      <c r="C73" t="s">
+        <v>376</v>
+      </c>
+      <c r="D73" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>116</v>
+      </c>
+      <c r="C74" t="s">
+        <v>75</v>
+      </c>
+      <c r="D74" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>122</v>
+      </c>
+      <c r="C75" t="s">
+        <v>364</v>
+      </c>
+      <c r="D75" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>120</v>
+      </c>
+      <c r="C76" t="s">
+        <v>97</v>
+      </c>
+      <c r="D76" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>124</v>
+      </c>
+      <c r="C77" t="s">
+        <v>19</v>
+      </c>
+      <c r="D77" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>126</v>
+      </c>
+      <c r="C78" t="s">
+        <v>37</v>
+      </c>
+      <c r="D78" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>118</v>
+      </c>
+      <c r="C79" t="s">
+        <v>64</v>
+      </c>
+      <c r="D79" t="s">
+        <v>375</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D60"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="50" customWidth="1"/>
+    <col min="3" max="4" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>377</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>378</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>379</v>
+      </c>
+      <c r="C4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>380</v>
+      </c>
+      <c r="C5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>381</v>
+      </c>
+      <c r="C6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>382</v>
+      </c>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>383</v>
+      </c>
+      <c r="C8" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>384</v>
+      </c>
+      <c r="C9" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>385</v>
+      </c>
+      <c r="C10" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>386</v>
+      </c>
+      <c r="C11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D11" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>387</v>
+      </c>
+      <c r="C12" t="s">
+        <v>3</v>
+      </c>
+      <c r="D12" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>388</v>
+      </c>
+      <c r="C13" t="s">
+        <v>3</v>
+      </c>
+      <c r="D13" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>378</v>
+      </c>
+      <c r="C14" t="s">
+        <v>3</v>
+      </c>
+      <c r="D14" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>381</v>
+      </c>
+      <c r="C15" t="s">
+        <v>3</v>
+      </c>
+      <c r="D15" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>379</v>
+      </c>
+      <c r="C16" t="s">
+        <v>3</v>
+      </c>
+      <c r="D16" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>380</v>
+      </c>
+      <c r="C17" t="s">
+        <v>3</v>
+      </c>
+      <c r="D17" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>381</v>
+      </c>
+      <c r="C18" t="s">
+        <v>3</v>
+      </c>
+      <c r="D18" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>378</v>
+      </c>
+      <c r="C19" t="s">
+        <v>3</v>
+      </c>
+      <c r="D19" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>379</v>
+      </c>
+      <c r="C20" t="s">
+        <v>3</v>
+      </c>
+      <c r="D20" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>382</v>
+      </c>
+      <c r="C21" t="s">
+        <v>19</v>
+      </c>
+      <c r="D21" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>377</v>
+      </c>
+      <c r="C22" t="s">
+        <v>3</v>
+      </c>
+      <c r="D22" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>381</v>
+      </c>
+      <c r="C23" t="s">
+        <v>3</v>
+      </c>
+      <c r="D23" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>378</v>
+      </c>
+      <c r="C24" t="s">
+        <v>3</v>
+      </c>
+      <c r="D24" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>377</v>
+      </c>
+      <c r="C25" t="s">
+        <v>3</v>
+      </c>
+      <c r="D25" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>379</v>
+      </c>
+      <c r="C26" t="s">
+        <v>3</v>
+      </c>
+      <c r="D26" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>380</v>
+      </c>
+      <c r="C27" t="s">
+        <v>3</v>
+      </c>
+      <c r="D27" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>380</v>
+      </c>
+      <c r="C28" t="s">
+        <v>3</v>
+      </c>
+      <c r="D28" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>381</v>
+      </c>
+      <c r="C29" t="s">
+        <v>3</v>
+      </c>
+      <c r="D29" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>378</v>
+      </c>
+      <c r="C30" t="s">
+        <v>3</v>
+      </c>
+      <c r="D30" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>381</v>
+      </c>
+      <c r="C31" t="s">
+        <v>3</v>
+      </c>
+      <c r="D31" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>380</v>
+      </c>
+      <c r="C32" t="s">
+        <v>3</v>
+      </c>
+      <c r="D32" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>379</v>
+      </c>
+      <c r="C33" t="s">
+        <v>3</v>
+      </c>
+      <c r="D33" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>377</v>
+      </c>
+      <c r="C34" t="s">
+        <v>3</v>
+      </c>
+      <c r="D34" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>377</v>
+      </c>
+      <c r="C35" t="s">
+        <v>3</v>
+      </c>
+      <c r="D35" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>378</v>
+      </c>
+      <c r="C36" t="s">
+        <v>3</v>
+      </c>
+      <c r="D36" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>377</v>
+      </c>
+      <c r="C37" t="s">
+        <v>3</v>
+      </c>
+      <c r="D37" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>378</v>
+      </c>
+      <c r="C38" t="s">
+        <v>3</v>
+      </c>
+      <c r="D38" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>378</v>
+      </c>
+      <c r="C39" t="s">
+        <v>3</v>
+      </c>
+      <c r="D39" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>379</v>
+      </c>
+      <c r="C40" t="s">
+        <v>3</v>
+      </c>
+      <c r="D40" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>378</v>
+      </c>
+      <c r="C41" t="s">
+        <v>97</v>
+      </c>
+      <c r="D41" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>377</v>
+      </c>
+      <c r="C42" t="s">
+        <v>3</v>
+      </c>
+      <c r="D42" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>379</v>
+      </c>
+      <c r="C43" t="s">
+        <v>3</v>
+      </c>
+      <c r="D43" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>382</v>
+      </c>
+      <c r="C44" t="s">
+        <v>75</v>
+      </c>
+      <c r="D44" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>380</v>
+      </c>
+      <c r="C45" t="s">
+        <v>3</v>
+      </c>
+      <c r="D45" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>381</v>
+      </c>
+      <c r="C46" t="s">
+        <v>3</v>
+      </c>
+      <c r="D46" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>383</v>
+      </c>
+      <c r="C47" t="s">
+        <v>3</v>
+      </c>
+      <c r="D47" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>379</v>
+      </c>
+      <c r="C48" t="s">
+        <v>3</v>
+      </c>
+      <c r="D48" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>377</v>
+      </c>
+      <c r="C49" t="s">
+        <v>3</v>
+      </c>
+      <c r="D49" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>378</v>
+      </c>
+      <c r="C50" t="s">
+        <v>19</v>
+      </c>
+      <c r="D50" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>379</v>
+      </c>
+      <c r="C51" t="s">
+        <v>30</v>
+      </c>
+      <c r="D51" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>380</v>
+      </c>
+      <c r="C52" t="s">
+        <v>3</v>
+      </c>
+      <c r="D52" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>381</v>
+      </c>
+      <c r="C53" t="s">
+        <v>28</v>
+      </c>
+      <c r="D53" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>382</v>
+      </c>
+      <c r="C54" t="s">
+        <v>19</v>
+      </c>
+      <c r="D54" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>383</v>
+      </c>
+      <c r="C55" t="s">
+        <v>3</v>
+      </c>
+      <c r="D55" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>384</v>
+      </c>
+      <c r="C56" t="s">
+        <v>3</v>
+      </c>
+      <c r="D56" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>385</v>
+      </c>
+      <c r="C57" t="s">
+        <v>3</v>
+      </c>
+      <c r="D57" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>386</v>
+      </c>
+      <c r="C58" t="s">
+        <v>3</v>
+      </c>
+      <c r="D58" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>387</v>
+      </c>
+      <c r="C59" t="s">
+        <v>3</v>
+      </c>
+      <c r="D59" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>388</v>
+      </c>
+      <c r="C60" t="s">
+        <v>3</v>
+      </c>
+      <c r="D60" t="s">
+        <v>375</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Stabilize Whois Intelligence Dashboard and Enhance Keyword Explorer with Intent Filters
</commit_message>
<xml_diff>
--- a/backend/rankings.xlsx
+++ b/backend/rankings.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4953" uniqueCount="389">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4989" uniqueCount="390">
   <si>
     <t>Keyword / Date</t>
   </si>
@@ -1188,6 +1188,9 @@
   </si>
   <si>
     <t>roof restoration cranbourne</t>
+  </si>
+  <si>
+    <t>2026-05-04</t>
   </si>
 </sst>
 </file>
@@ -2543,7 +2546,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D72"/>
+  <dimension ref="A1:D84"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -3344,6 +3347,138 @@
       </c>
       <c r="D72" t="s">
         <v>375</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>377</v>
+      </c>
+      <c r="C73" t="s">
+        <v>3</v>
+      </c>
+      <c r="D73" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>378</v>
+      </c>
+      <c r="C74" t="s">
+        <v>97</v>
+      </c>
+      <c r="D74" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>379</v>
+      </c>
+      <c r="C75" t="s">
+        <v>19</v>
+      </c>
+      <c r="D75" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>380</v>
+      </c>
+      <c r="C76" t="s">
+        <v>3</v>
+      </c>
+      <c r="D76" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>381</v>
+      </c>
+      <c r="C77" t="s">
+        <v>3</v>
+      </c>
+      <c r="D77" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>382</v>
+      </c>
+      <c r="C78" t="s">
+        <v>19</v>
+      </c>
+      <c r="D78" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>383</v>
+      </c>
+      <c r="C79" t="s">
+        <v>3</v>
+      </c>
+      <c r="D79" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>384</v>
+      </c>
+      <c r="C80" t="s">
+        <v>3</v>
+      </c>
+      <c r="D80" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>385</v>
+      </c>
+      <c r="C81" t="s">
+        <v>3</v>
+      </c>
+      <c r="D81" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>386</v>
+      </c>
+      <c r="C82" t="s">
+        <v>3</v>
+      </c>
+      <c r="D82" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>387</v>
+      </c>
+      <c r="C83" t="s">
+        <v>3</v>
+      </c>
+      <c r="D83" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>388</v>
+      </c>
+      <c r="C84" t="s">
+        <v>3</v>
+      </c>
+      <c r="D84" t="s">
+        <v>389</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🚀 PRODUCTION SYNC: Enterprise SEO & UI Updates
</commit_message>
<xml_diff>
--- a/backend/rankings.xlsx
+++ b/backend/rankings.xlsx
@@ -15,13 +15,14 @@
     <sheet sheetId="9" name="abc.con" state="visible" r:id="rId12"/>
     <sheet sheetId="10" name="adamdental.com.au" state="visible" r:id="rId13"/>
     <sheet sheetId="11" name="challengebricksandroofing.com.a" state="visible" r:id="rId14"/>
+    <sheet sheetId="12" name="melbournedjhire" state="visible" r:id="rId15"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4989" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5173" uniqueCount="395">
   <si>
     <t>Keyword / Date</t>
   </si>
@@ -1191,6 +1192,21 @@
   </si>
   <si>
     <t>2026-05-04</t>
+  </si>
+  <si>
+    <t>2026-05-06</t>
+  </si>
+  <si>
+    <t>1//10 LL 1</t>
+  </si>
+  <si>
+    <t>1//4 LL 1</t>
+  </si>
+  <si>
+    <t>1//3 LL 1</t>
+  </si>
+  <si>
+    <t>1//6 LL 1</t>
   </si>
 </sst>
 </file>
@@ -3487,6 +3503,696 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D61"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="50" customWidth="1"/>
+    <col min="3" max="4" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D2" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C3" t="s">
+        <v>64</v>
+      </c>
+      <c r="D3" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C5" t="s">
+        <v>97</v>
+      </c>
+      <c r="D5" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C6" t="s">
+        <v>367</v>
+      </c>
+      <c r="D6" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>70</v>
+      </c>
+      <c r="C7" t="s">
+        <v>391</v>
+      </c>
+      <c r="D7" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>73</v>
+      </c>
+      <c r="C8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D8" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C9" t="s">
+        <v>392</v>
+      </c>
+      <c r="D9" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>76</v>
+      </c>
+      <c r="C10" t="s">
+        <v>367</v>
+      </c>
+      <c r="D10" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>77</v>
+      </c>
+      <c r="C11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D11" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>78</v>
+      </c>
+      <c r="C12" t="s">
+        <v>64</v>
+      </c>
+      <c r="D12" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C13" t="s">
+        <v>64</v>
+      </c>
+      <c r="D13" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>80</v>
+      </c>
+      <c r="C14" t="s">
+        <v>64</v>
+      </c>
+      <c r="D14" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C15" t="s">
+        <v>64</v>
+      </c>
+      <c r="D15" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>82</v>
+      </c>
+      <c r="C16" t="s">
+        <v>3</v>
+      </c>
+      <c r="D16" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>85</v>
+      </c>
+      <c r="C17" t="s">
+        <v>393</v>
+      </c>
+      <c r="D17" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>86</v>
+      </c>
+      <c r="C18" t="s">
+        <v>392</v>
+      </c>
+      <c r="D18" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>87</v>
+      </c>
+      <c r="C19" t="s">
+        <v>391</v>
+      </c>
+      <c r="D19" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>89</v>
+      </c>
+      <c r="C20" t="s">
+        <v>3</v>
+      </c>
+      <c r="D20" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>91</v>
+      </c>
+      <c r="C21" t="s">
+        <v>14</v>
+      </c>
+      <c r="D21" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C22" t="s">
+        <v>64</v>
+      </c>
+      <c r="D22" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>65</v>
+      </c>
+      <c r="C23" t="s">
+        <v>64</v>
+      </c>
+      <c r="D23" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>66</v>
+      </c>
+      <c r="C24" t="s">
+        <v>64</v>
+      </c>
+      <c r="D24" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>68</v>
+      </c>
+      <c r="C25" t="s">
+        <v>64</v>
+      </c>
+      <c r="D25" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>60</v>
+      </c>
+      <c r="C26" t="s">
+        <v>392</v>
+      </c>
+      <c r="D26" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>70</v>
+      </c>
+      <c r="C27" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>73</v>
+      </c>
+      <c r="C28" t="s">
+        <v>64</v>
+      </c>
+      <c r="D28" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>74</v>
+      </c>
+      <c r="C29" t="s">
+        <v>392</v>
+      </c>
+      <c r="D29" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>76</v>
+      </c>
+      <c r="C30" t="s">
+        <v>393</v>
+      </c>
+      <c r="D30" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>77</v>
+      </c>
+      <c r="C31" t="s">
+        <v>394</v>
+      </c>
+      <c r="D31" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>78</v>
+      </c>
+      <c r="C32" t="s">
+        <v>64</v>
+      </c>
+      <c r="D32" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>79</v>
+      </c>
+      <c r="C33" t="s">
+        <v>64</v>
+      </c>
+      <c r="D33" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>80</v>
+      </c>
+      <c r="C34" t="s">
+        <v>64</v>
+      </c>
+      <c r="D34" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>81</v>
+      </c>
+      <c r="C35" t="s">
+        <v>64</v>
+      </c>
+      <c r="D35" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>82</v>
+      </c>
+      <c r="C36" t="s">
+        <v>3</v>
+      </c>
+      <c r="D36" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>85</v>
+      </c>
+      <c r="C37" t="s">
+        <v>3</v>
+      </c>
+      <c r="D37" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>86</v>
+      </c>
+      <c r="C38" t="s">
+        <v>367</v>
+      </c>
+      <c r="D38" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>87</v>
+      </c>
+      <c r="C39" t="s">
+        <v>393</v>
+      </c>
+      <c r="D39" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>89</v>
+      </c>
+      <c r="C40" t="s">
+        <v>3</v>
+      </c>
+      <c r="D40" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>91</v>
+      </c>
+      <c r="C41" t="s">
+        <v>14</v>
+      </c>
+      <c r="D41" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>63</v>
+      </c>
+      <c r="C42" t="s">
+        <v>64</v>
+      </c>
+      <c r="D42" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>65</v>
+      </c>
+      <c r="C43" t="s">
+        <v>64</v>
+      </c>
+      <c r="D43" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>66</v>
+      </c>
+      <c r="C44" t="s">
+        <v>64</v>
+      </c>
+      <c r="D44" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>68</v>
+      </c>
+      <c r="C45" t="s">
+        <v>64</v>
+      </c>
+      <c r="D45" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>60</v>
+      </c>
+      <c r="C46" t="s">
+        <v>367</v>
+      </c>
+      <c r="D46" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>70</v>
+      </c>
+      <c r="C47" t="s">
+        <v>391</v>
+      </c>
+      <c r="D47" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="C48" t="s">
+        <v>64</v>
+      </c>
+      <c r="D48" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="C49" t="s">
+        <v>3</v>
+      </c>
+      <c r="D49" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="C50" t="s">
+        <v>394</v>
+      </c>
+      <c r="D50" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="C51" t="s">
+        <v>394</v>
+      </c>
+      <c r="D51" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="C52" t="s">
+        <v>64</v>
+      </c>
+      <c r="D52" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="C54" t="s">
+        <v>64</v>
+      </c>
+      <c r="D54" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="C55" t="s">
+        <v>64</v>
+      </c>
+      <c r="D55" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="C56" t="s">
+        <v>367</v>
+      </c>
+      <c r="D56" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>85</v>
+      </c>
+      <c r="C57" t="s">
+        <v>393</v>
+      </c>
+      <c r="D57" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>86</v>
+      </c>
+      <c r="C58" t="s">
+        <v>64</v>
+      </c>
+      <c r="D58" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>87</v>
+      </c>
+      <c r="C59" t="s">
+        <v>391</v>
+      </c>
+      <c r="D59" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>89</v>
+      </c>
+      <c r="C60" t="s">
+        <v>3</v>
+      </c>
+      <c r="D60" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>91</v>
+      </c>
+      <c r="C61" t="s">
+        <v>391</v>
+      </c>
+      <c r="D61" t="s">
+        <v>390</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C9"/>

</xml_diff>